<commit_message>
Prise en compte du retour de test
</commit_message>
<xml_diff>
--- a/docs/Cartes-a-jouer--repartition.xlsx
+++ b/docs/Cartes-a-jouer--repartition.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\leand\Documents\GitHub\Donjons-et-Barons\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE275B44-DDE6-4D0D-AA21-992D35776967}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BE00268-0D8E-4B90-AEAE-D1A92F99FB85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-9120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -234,7 +234,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="14">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -393,12 +393,30 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -466,11 +484,35 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -489,18 +531,6 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -519,13 +549,31 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1771,203 +1819,300 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1E300F5-BB8C-42D4-B150-781935673603}">
-  <dimension ref="B2:F15"/>
+  <dimension ref="B2:G15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.5703125" customWidth="1"/>
     <col min="2" max="2" width="23.7109375" customWidth="1"/>
     <col min="3" max="3" width="8.7109375" customWidth="1"/>
-    <col min="4" max="6" width="5.7109375" customWidth="1"/>
+    <col min="4" max="7" width="4.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B2" s="21" t="s">
         <v>36</v>
       </c>
       <c r="C2" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="23" t="s">
+      <c r="D2" s="24" t="s">
         <v>37</v>
       </c>
-      <c r="E2" s="24"/>
+      <c r="E2" s="47"/>
       <c r="F2" s="25"/>
-    </row>
-    <row r="3" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="G2" s="26"/>
+    </row>
+    <row r="3" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3" s="18" t="s">
         <v>12</v>
       </c>
       <c r="C3" s="18">
-        <v>6</v>
-      </c>
-      <c r="D3" s="26">
+        <v>4</v>
+      </c>
+      <c r="D3" s="34">
         <f>SUM(C3:C5)</f>
-        <v>18</v>
-      </c>
-      <c r="E3" s="27"/>
-      <c r="F3" s="42">
+        <v>15</v>
+      </c>
+      <c r="E3" s="48"/>
+      <c r="F3" s="35"/>
+      <c r="G3" s="31">
         <f>SUM(C3:C15)</f>
         <v>40</v>
       </c>
     </row>
-    <row r="4" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B4" s="18" t="s">
         <v>13</v>
       </c>
       <c r="C4" s="18">
-        <v>6</v>
-      </c>
-      <c r="D4" s="28"/>
-      <c r="E4" s="29"/>
-      <c r="F4" s="43"/>
-    </row>
-    <row r="5" spans="2:6" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+      <c r="D4" s="36"/>
+      <c r="E4" s="49"/>
+      <c r="F4" s="37"/>
+      <c r="G4" s="32"/>
+    </row>
+    <row r="5" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B5" s="18" t="s">
         <v>14</v>
       </c>
       <c r="C5" s="18">
         <v>6</v>
       </c>
-      <c r="D5" s="30"/>
-      <c r="E5" s="31"/>
-      <c r="F5" s="43"/>
-    </row>
-    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="D5" s="38"/>
+      <c r="E5" s="50"/>
+      <c r="F5" s="39"/>
+      <c r="G5" s="32"/>
+    </row>
+    <row r="6" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B6" s="20" t="s">
         <v>16</v>
       </c>
       <c r="C6" s="20">
         <v>2</v>
       </c>
-      <c r="D6" s="32">
+      <c r="D6" s="27">
         <f>SUM(C6:C8)</f>
-        <v>6</v>
-      </c>
-      <c r="E6" s="33">
+        <v>9</v>
+      </c>
+      <c r="E6" s="27">
+        <f>D6+D9</f>
+        <v>15</v>
+      </c>
+      <c r="F6" s="30">
         <f>SUM(C6:C11)</f>
-        <v>18</v>
-      </c>
-      <c r="F6" s="43"/>
-    </row>
-    <row r="7" spans="2:6" x14ac:dyDescent="0.25">
+        <v>21</v>
+      </c>
+      <c r="G6" s="32"/>
+    </row>
+    <row r="7" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B7" s="20" t="s">
         <v>18</v>
       </c>
       <c r="C7" s="20">
-        <v>2</v>
-      </c>
-      <c r="D7" s="34"/>
-      <c r="E7" s="33"/>
-      <c r="F7" s="43"/>
-    </row>
-    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+      <c r="D7" s="28"/>
+      <c r="E7" s="54"/>
+      <c r="F7" s="30"/>
+      <c r="G7" s="32"/>
+    </row>
+    <row r="8" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B8" s="20" t="s">
         <v>17</v>
       </c>
       <c r="C8" s="20">
-        <v>2</v>
-      </c>
-      <c r="D8" s="35"/>
-      <c r="E8" s="33"/>
-      <c r="F8" s="43"/>
-    </row>
-    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+      <c r="D8" s="29"/>
+      <c r="E8" s="54"/>
+      <c r="F8" s="30"/>
+      <c r="G8" s="32"/>
+    </row>
+    <row r="9" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B9" s="20" t="s">
-        <v>38</v>
+        <v>8</v>
       </c>
       <c r="C9" s="20">
+        <v>3</v>
+      </c>
+      <c r="D9" s="27">
+        <f>SUM(C9:C10)</f>
         <v>6</v>
       </c>
-      <c r="D9" s="20">
-        <f>C9</f>
-        <v>6</v>
-      </c>
-      <c r="E9" s="33"/>
-      <c r="F9" s="43"/>
-    </row>
-    <row r="10" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="E9" s="54"/>
+      <c r="F9" s="30"/>
+      <c r="G9" s="32"/>
+    </row>
+    <row r="10" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B10" s="20" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C10" s="20">
         <v>3</v>
       </c>
-      <c r="D10" s="32">
-        <f>SUM(C10:C11)</f>
+      <c r="D10" s="46"/>
+      <c r="E10" s="46"/>
+      <c r="F10" s="30"/>
+      <c r="G10" s="32"/>
+    </row>
+    <row r="11" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B11" s="20" t="s">
+        <v>38</v>
+      </c>
+      <c r="C11" s="20">
         <v>6</v>
       </c>
-      <c r="E10" s="33"/>
-      <c r="F10" s="43"/>
-    </row>
-    <row r="11" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B11" s="20" t="s">
-        <v>7</v>
-      </c>
-      <c r="C11" s="20">
-        <v>3</v>
-      </c>
-      <c r="D11" s="35"/>
-      <c r="E11" s="33"/>
-      <c r="F11" s="43"/>
-    </row>
-    <row r="12" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="D11" s="23">
+        <f>C11</f>
+        <v>6</v>
+      </c>
+      <c r="E11" s="23">
+        <f>D11</f>
+        <v>6</v>
+      </c>
+      <c r="F11" s="30"/>
+      <c r="G11" s="32"/>
+    </row>
+    <row r="12" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B12" s="18" t="s">
         <v>9</v>
       </c>
       <c r="C12" s="18">
         <v>1</v>
       </c>
-      <c r="D12" s="36">
+      <c r="D12" s="40">
         <f>SUM(C12:C15)</f>
         <v>4</v>
       </c>
-      <c r="E12" s="37"/>
-      <c r="F12" s="43"/>
-    </row>
-    <row r="13" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="E12" s="51"/>
+      <c r="F12" s="41"/>
+      <c r="G12" s="32"/>
+    </row>
+    <row r="13" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B13" s="18" t="s">
         <v>35</v>
       </c>
       <c r="C13" s="18">
         <v>1</v>
       </c>
-      <c r="D13" s="38"/>
-      <c r="E13" s="39"/>
+      <c r="D13" s="42"/>
+      <c r="E13" s="52"/>
       <c r="F13" s="43"/>
-    </row>
-    <row r="14" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="G13" s="32"/>
+    </row>
+    <row r="14" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B14" s="18" t="s">
         <v>11</v>
       </c>
       <c r="C14" s="18">
         <v>1</v>
       </c>
-      <c r="D14" s="38"/>
-      <c r="E14" s="39"/>
+      <c r="D14" s="42"/>
+      <c r="E14" s="52"/>
       <c r="F14" s="43"/>
-    </row>
-    <row r="15" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="G14" s="32"/>
+    </row>
+    <row r="15" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B15" s="22" t="s">
         <v>39</v>
       </c>
       <c r="C15" s="18">
         <v>1</v>
       </c>
-      <c r="D15" s="40"/>
-      <c r="E15" s="41"/>
-      <c r="F15" s="44"/>
+      <c r="D15" s="44"/>
+      <c r="E15" s="53"/>
+      <c r="F15" s="45"/>
+      <c r="G15" s="33"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="D2:F2"/>
+  <mergeCells count="8">
+    <mergeCell ref="D2:G2"/>
     <mergeCell ref="D6:D8"/>
-    <mergeCell ref="D10:D11"/>
-    <mergeCell ref="E6:E11"/>
-    <mergeCell ref="F3:F15"/>
-    <mergeCell ref="D3:E5"/>
-    <mergeCell ref="D12:E15"/>
+    <mergeCell ref="F6:F11"/>
+    <mergeCell ref="G3:G15"/>
+    <mergeCell ref="D3:F5"/>
+    <mergeCell ref="D12:F15"/>
+    <mergeCell ref="D9:D10"/>
+    <mergeCell ref="E6:E10"/>
   </mergeCells>
   <conditionalFormatting sqref="C3:C5">
+    <cfRule type="colorScale" priority="25">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF5A8AC6"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C3:C8 C12:C15">
+    <cfRule type="colorScale" priority="18">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEF9C"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="19">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF5A8AC6"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C6:C8">
+    <cfRule type="colorScale" priority="24">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF5A8AC6"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C12:C15">
+    <cfRule type="colorScale" priority="20">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF5A8AC6"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C9:C10">
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEF9C"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="6">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FF5A8AC6"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C9">
     <cfRule type="colorScale" priority="8">
       <colorScale>
         <cfvo type="min"/>
@@ -1979,7 +2124,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C6:C8">
+  <conditionalFormatting sqref="C10">
     <cfRule type="colorScale" priority="7">
       <colorScale>
         <cfvo type="min"/>
@@ -1991,20 +2136,16 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C9">
-    <cfRule type="colorScale" priority="6">
+  <conditionalFormatting sqref="C11">
+    <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
         <cfvo type="max"/>
-        <color rgb="FF5A8AC6"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FFF8696B"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEF9C"/>
       </colorScale>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C10">
-    <cfRule type="colorScale" priority="5">
+    <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -2027,29 +2168,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C12:C15">
-    <cfRule type="colorScale" priority="3">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF5A8AC6"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="C3:C15">
-    <cfRule type="colorScale" priority="2">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF5A8AC6"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -2062,7 +2181,7 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <ignoredErrors>
-    <ignoredError sqref="D6:E6 D10 D12 D3" formulaRange="1"/>
+    <ignoredError sqref="F6 D12 D3 D9 D6" formulaRange="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Mise à jour des cartes suite au test
</commit_message>
<xml_diff>
--- a/docs/Cartes-a-jouer--repartition.xlsx
+++ b/docs/Cartes-a-jouer--repartition.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\leand\Documents\GitHub\Donjons-et-Barons\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BE00268-0D8E-4B90-AEAE-D1A92F99FB85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA478273-47E7-4304-AF66-8205D3E32C20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-9120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -490,6 +490,9 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -516,61 +519,58 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1838,9 +1838,9 @@
       <c r="D2" s="24" t="s">
         <v>37</v>
       </c>
-      <c r="E2" s="47"/>
-      <c r="F2" s="25"/>
-      <c r="G2" s="26"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="26"/>
+      <c r="G2" s="27"/>
     </row>
     <row r="3" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B3" s="18" t="s">
@@ -1849,13 +1849,13 @@
       <c r="C3" s="18">
         <v>4</v>
       </c>
-      <c r="D3" s="34">
+      <c r="D3" s="35">
         <f>SUM(C3:C5)</f>
         <v>15</v>
       </c>
-      <c r="E3" s="48"/>
-      <c r="F3" s="35"/>
-      <c r="G3" s="31">
+      <c r="E3" s="36"/>
+      <c r="F3" s="37"/>
+      <c r="G3" s="32">
         <f>SUM(C3:C15)</f>
         <v>40</v>
       </c>
@@ -1867,10 +1867,10 @@
       <c r="C4" s="18">
         <v>5</v>
       </c>
-      <c r="D4" s="36"/>
-      <c r="E4" s="49"/>
-      <c r="F4" s="37"/>
-      <c r="G4" s="32"/>
+      <c r="D4" s="38"/>
+      <c r="E4" s="39"/>
+      <c r="F4" s="40"/>
+      <c r="G4" s="33"/>
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B5" s="18" t="s">
@@ -1879,10 +1879,10 @@
       <c r="C5" s="18">
         <v>6</v>
       </c>
-      <c r="D5" s="38"/>
-      <c r="E5" s="50"/>
-      <c r="F5" s="39"/>
-      <c r="G5" s="32"/>
+      <c r="D5" s="41"/>
+      <c r="E5" s="42"/>
+      <c r="F5" s="43"/>
+      <c r="G5" s="33"/>
     </row>
     <row r="6" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B6" s="20" t="s">
@@ -1891,19 +1891,19 @@
       <c r="C6" s="20">
         <v>2</v>
       </c>
-      <c r="D6" s="27">
+      <c r="D6" s="28">
         <f>SUM(C6:C8)</f>
         <v>9</v>
       </c>
-      <c r="E6" s="27">
+      <c r="E6" s="28">
         <f>D6+D9</f>
         <v>15</v>
       </c>
-      <c r="F6" s="30">
+      <c r="F6" s="31">
         <f>SUM(C6:C11)</f>
         <v>21</v>
       </c>
-      <c r="G6" s="32"/>
+      <c r="G6" s="33"/>
     </row>
     <row r="7" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B7" s="20" t="s">
@@ -1912,10 +1912,10 @@
       <c r="C7" s="20">
         <v>3</v>
       </c>
-      <c r="D7" s="28"/>
+      <c r="D7" s="29"/>
       <c r="E7" s="54"/>
-      <c r="F7" s="30"/>
-      <c r="G7" s="32"/>
+      <c r="F7" s="31"/>
+      <c r="G7" s="33"/>
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B8" s="20" t="s">
@@ -1924,10 +1924,10 @@
       <c r="C8" s="20">
         <v>4</v>
       </c>
-      <c r="D8" s="29"/>
+      <c r="D8" s="30"/>
       <c r="E8" s="54"/>
-      <c r="F8" s="30"/>
-      <c r="G8" s="32"/>
+      <c r="F8" s="31"/>
+      <c r="G8" s="33"/>
     </row>
     <row r="9" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B9" s="20" t="s">
@@ -1936,13 +1936,13 @@
       <c r="C9" s="20">
         <v>3</v>
       </c>
-      <c r="D9" s="27">
+      <c r="D9" s="28">
         <f>SUM(C9:C10)</f>
         <v>6</v>
       </c>
       <c r="E9" s="54"/>
-      <c r="F9" s="30"/>
-      <c r="G9" s="32"/>
+      <c r="F9" s="31"/>
+      <c r="G9" s="33"/>
     </row>
     <row r="10" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B10" s="20" t="s">
@@ -1951,10 +1951,10 @@
       <c r="C10" s="20">
         <v>3</v>
       </c>
-      <c r="D10" s="46"/>
-      <c r="E10" s="46"/>
-      <c r="F10" s="30"/>
-      <c r="G10" s="32"/>
+      <c r="D10" s="53"/>
+      <c r="E10" s="53"/>
+      <c r="F10" s="31"/>
+      <c r="G10" s="33"/>
     </row>
     <row r="11" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B11" s="20" t="s">
@@ -1971,8 +1971,8 @@
         <f>D11</f>
         <v>6</v>
       </c>
-      <c r="F11" s="30"/>
-      <c r="G11" s="32"/>
+      <c r="F11" s="31"/>
+      <c r="G11" s="33"/>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B12" s="18" t="s">
@@ -1981,13 +1981,13 @@
       <c r="C12" s="18">
         <v>1</v>
       </c>
-      <c r="D12" s="40">
+      <c r="D12" s="44">
         <f>SUM(C12:C15)</f>
         <v>4</v>
       </c>
-      <c r="E12" s="51"/>
-      <c r="F12" s="41"/>
-      <c r="G12" s="32"/>
+      <c r="E12" s="45"/>
+      <c r="F12" s="46"/>
+      <c r="G12" s="33"/>
     </row>
     <row r="13" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B13" s="18" t="s">
@@ -1996,10 +1996,10 @@
       <c r="C13" s="18">
         <v>1</v>
       </c>
-      <c r="D13" s="42"/>
-      <c r="E13" s="52"/>
-      <c r="F13" s="43"/>
-      <c r="G13" s="32"/>
+      <c r="D13" s="47"/>
+      <c r="E13" s="48"/>
+      <c r="F13" s="49"/>
+      <c r="G13" s="33"/>
     </row>
     <row r="14" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B14" s="18" t="s">
@@ -2008,10 +2008,10 @@
       <c r="C14" s="18">
         <v>1</v>
       </c>
-      <c r="D14" s="42"/>
-      <c r="E14" s="52"/>
-      <c r="F14" s="43"/>
-      <c r="G14" s="32"/>
+      <c r="D14" s="47"/>
+      <c r="E14" s="48"/>
+      <c r="F14" s="49"/>
+      <c r="G14" s="33"/>
     </row>
     <row r="15" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B15" s="22" t="s">
@@ -2020,10 +2020,10 @@
       <c r="C15" s="18">
         <v>1</v>
       </c>
-      <c r="D15" s="44"/>
-      <c r="E15" s="53"/>
-      <c r="F15" s="45"/>
-      <c r="G15" s="33"/>
+      <c r="D15" s="50"/>
+      <c r="E15" s="51"/>
+      <c r="F15" s="52"/>
+      <c r="G15" s="34"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -2068,6 +2068,16 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="C3:C15">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF63BE7B"/>
+        <color rgb="FFFFEF9C"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="C6:C8">
     <cfRule type="colorScale" priority="24">
       <colorScale>
@@ -2080,8 +2090,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C12:C15">
-    <cfRule type="colorScale" priority="20">
+  <conditionalFormatting sqref="C9">
+    <cfRule type="colorScale" priority="8">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -2102,18 +2112,6 @@
       </colorScale>
     </cfRule>
     <cfRule type="colorScale" priority="6">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FF5A8AC6"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FFF8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C9">
-    <cfRule type="colorScale" priority="8">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -2155,8 +2153,6 @@
         <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C11">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
@@ -2168,13 +2164,15 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C3:C15">
-    <cfRule type="colorScale" priority="1">
+  <conditionalFormatting sqref="C12:C15">
+    <cfRule type="colorScale" priority="20">
       <colorScale>
         <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
         <cfvo type="max"/>
-        <color rgb="FF63BE7B"/>
-        <color rgb="FFFFEF9C"/>
+        <color rgb="FF5A8AC6"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FFF8696B"/>
       </colorScale>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Bonne avancée de la description des cartes Actions et des cartes Evénements
</commit_message>
<xml_diff>
--- a/docs/Cartes-a-jouer--repartition.xlsx
+++ b/docs/Cartes-a-jouer--repartition.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\leand\Documents\GitHub\Donjons-et-Barons\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA478273-47E7-4304-AF66-8205D3E32C20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{473A9276-0479-4E0B-8D8D-3B68F5A40A6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-9120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Répartition" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="42">
   <si>
     <t>Type</t>
   </si>
@@ -147,9 +147,6 @@
     <t>Recruter Chevalier</t>
   </si>
   <si>
-    <t>Carte</t>
-  </si>
-  <si>
     <t>Regroupements</t>
   </si>
   <si>
@@ -157,6 +154,15 @@
   </si>
   <si>
     <t>Complot à la Cour</t>
+  </si>
+  <si>
+    <t>Carte Action</t>
+  </si>
+  <si>
+    <t>Crédits</t>
+  </si>
+  <si>
+    <t>Exiler Chevalier</t>
   </si>
 </sst>
 </file>
@@ -190,7 +196,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -229,7 +235,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFC28D7C"/>
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-0.249977111117893"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -481,11 +493,11 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -507,13 +519,13 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1478,7 +1490,7 @@
     </row>
     <row r="10" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B10" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C10" s="2">
         <v>8</v>
@@ -1819,224 +1831,266 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E1E300F5-BB8C-42D4-B150-781935673603}">
-  <dimension ref="B2:G15"/>
+  <dimension ref="B2:H15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.5703125" customWidth="1"/>
     <col min="2" max="2" width="23.7109375" customWidth="1"/>
-    <col min="3" max="3" width="8.7109375" customWidth="1"/>
-    <col min="4" max="7" width="4.7109375" customWidth="1"/>
+    <col min="3" max="4" width="7.7109375" customWidth="1"/>
+    <col min="5" max="8" width="4.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B2" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="C2" s="21" t="s">
+        <v>40</v>
+      </c>
+      <c r="D2" s="21" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" s="24" t="s">
         <v>36</v>
       </c>
-      <c r="C2" s="21" t="s">
-        <v>5</v>
-      </c>
-      <c r="D2" s="24" t="s">
-        <v>37</v>
-      </c>
-      <c r="E2" s="25"/>
-      <c r="F2" s="26"/>
-      <c r="G2" s="27"/>
-    </row>
-    <row r="3" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="F2" s="25"/>
+      <c r="G2" s="26"/>
+      <c r="H2" s="27"/>
+    </row>
+    <row r="3" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B3" s="18" t="s">
         <v>12</v>
       </c>
       <c r="C3" s="18">
+        <v>3</v>
+      </c>
+      <c r="D3" s="18">
         <v>4</v>
       </c>
-      <c r="D3" s="35">
-        <f>SUM(C3:C5)</f>
+      <c r="E3" s="35">
+        <f>SUM(D3:D5)</f>
         <v>15</v>
       </c>
-      <c r="E3" s="36"/>
-      <c r="F3" s="37"/>
-      <c r="G3" s="32">
-        <f>SUM(C3:C15)</f>
+      <c r="F3" s="36"/>
+      <c r="G3" s="37"/>
+      <c r="H3" s="32">
+        <f>SUM(D3:D15)</f>
         <v>40</v>
       </c>
     </row>
-    <row r="4" spans="2:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B4" s="18" t="s">
         <v>13</v>
       </c>
       <c r="C4" s="18">
+        <v>2</v>
+      </c>
+      <c r="D4" s="18">
         <v>5</v>
       </c>
-      <c r="D4" s="38"/>
-      <c r="E4" s="39"/>
-      <c r="F4" s="40"/>
-      <c r="G4" s="33"/>
-    </row>
-    <row r="5" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="E4" s="38"/>
+      <c r="F4" s="39"/>
+      <c r="G4" s="40"/>
+      <c r="H4" s="33"/>
+    </row>
+    <row r="5" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B5" s="18" t="s">
         <v>14</v>
       </c>
       <c r="C5" s="18">
+        <v>1</v>
+      </c>
+      <c r="D5" s="18">
         <v>6</v>
       </c>
-      <c r="D5" s="41"/>
-      <c r="E5" s="42"/>
-      <c r="F5" s="43"/>
-      <c r="G5" s="33"/>
-    </row>
-    <row r="6" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="E5" s="41"/>
+      <c r="F5" s="42"/>
+      <c r="G5" s="43"/>
+      <c r="H5" s="33"/>
+    </row>
+    <row r="6" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B6" s="20" t="s">
         <v>16</v>
       </c>
       <c r="C6" s="20">
+        <v>3</v>
+      </c>
+      <c r="D6" s="20">
         <v>2</v>
       </c>
-      <c r="D6" s="28">
-        <f>SUM(C6:C8)</f>
+      <c r="E6" s="28">
+        <f>SUM(D6:D8)</f>
         <v>9</v>
       </c>
-      <c r="E6" s="28">
-        <f>D6+D9</f>
+      <c r="F6" s="28">
+        <f>E6+E9</f>
         <v>15</v>
       </c>
-      <c r="F6" s="31">
-        <f>SUM(C6:C11)</f>
+      <c r="G6" s="31">
+        <f>SUM(D6:D11)</f>
         <v>21</v>
       </c>
-      <c r="G6" s="33"/>
-    </row>
-    <row r="7" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="H6" s="33"/>
+    </row>
+    <row r="7" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B7" s="20" t="s">
         <v>18</v>
       </c>
       <c r="C7" s="20">
+        <v>2</v>
+      </c>
+      <c r="D7" s="20">
         <v>3</v>
       </c>
-      <c r="D7" s="29"/>
-      <c r="E7" s="54"/>
-      <c r="F7" s="31"/>
-      <c r="G7" s="33"/>
-    </row>
-    <row r="8" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="E7" s="29"/>
+      <c r="F7" s="54"/>
+      <c r="G7" s="31"/>
+      <c r="H7" s="33"/>
+    </row>
+    <row r="8" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B8" s="20" t="s">
         <v>17</v>
       </c>
       <c r="C8" s="20">
+        <v>1</v>
+      </c>
+      <c r="D8" s="20">
         <v>4</v>
       </c>
-      <c r="D8" s="30"/>
-      <c r="E8" s="54"/>
-      <c r="F8" s="31"/>
-      <c r="G8" s="33"/>
-    </row>
-    <row r="9" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="E8" s="30"/>
+      <c r="F8" s="54"/>
+      <c r="G8" s="31"/>
+      <c r="H8" s="33"/>
+    </row>
+    <row r="9" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B9" s="20" t="s">
         <v>8</v>
       </c>
       <c r="C9" s="20">
+        <v>1</v>
+      </c>
+      <c r="D9" s="20">
         <v>3</v>
       </c>
-      <c r="D9" s="28">
-        <f>SUM(C9:C10)</f>
+      <c r="E9" s="28">
+        <f>SUM(D9:D10)</f>
         <v>6</v>
       </c>
-      <c r="E9" s="54"/>
-      <c r="F9" s="31"/>
-      <c r="G9" s="33"/>
-    </row>
-    <row r="10" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="F9" s="54"/>
+      <c r="G9" s="31"/>
+      <c r="H9" s="33"/>
+    </row>
+    <row r="10" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B10" s="20" t="s">
         <v>7</v>
       </c>
       <c r="C10" s="20">
+        <v>1</v>
+      </c>
+      <c r="D10" s="20">
         <v>3</v>
       </c>
-      <c r="D10" s="53"/>
       <c r="E10" s="53"/>
-      <c r="F10" s="31"/>
-      <c r="G10" s="33"/>
-    </row>
-    <row r="11" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="F10" s="53"/>
+      <c r="G10" s="31"/>
+      <c r="H10" s="33"/>
+    </row>
+    <row r="11" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B11" s="20" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C11" s="20">
+        <v>3</v>
+      </c>
+      <c r="D11" s="20">
         <v>6</v>
       </c>
-      <c r="D11" s="23">
-        <f>C11</f>
-        <v>6</v>
-      </c>
-      <c r="E11" s="23">
+      <c r="E11" s="22">
         <f>D11</f>
         <v>6</v>
       </c>
-      <c r="F11" s="31"/>
-      <c r="G11" s="33"/>
-    </row>
-    <row r="12" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="F11" s="22">
+        <f>E11</f>
+        <v>6</v>
+      </c>
+      <c r="G11" s="31"/>
+      <c r="H11" s="33"/>
+    </row>
+    <row r="12" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B12" s="18" t="s">
         <v>9</v>
       </c>
       <c r="C12" s="18">
+        <v>3</v>
+      </c>
+      <c r="D12" s="18">
         <v>1</v>
       </c>
-      <c r="D12" s="44">
-        <f>SUM(C12:C15)</f>
+      <c r="E12" s="44">
+        <f>SUM(D12:D15)</f>
         <v>4</v>
       </c>
-      <c r="E12" s="45"/>
-      <c r="F12" s="46"/>
-      <c r="G12" s="33"/>
-    </row>
-    <row r="13" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="F12" s="45"/>
+      <c r="G12" s="46"/>
+      <c r="H12" s="33"/>
+    </row>
+    <row r="13" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B13" s="18" t="s">
         <v>35</v>
       </c>
       <c r="C13" s="18">
+        <v>3</v>
+      </c>
+      <c r="D13" s="18">
         <v>1</v>
       </c>
-      <c r="D13" s="47"/>
-      <c r="E13" s="48"/>
-      <c r="F13" s="49"/>
-      <c r="G13" s="33"/>
-    </row>
-    <row r="14" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="E13" s="47"/>
+      <c r="F13" s="48"/>
+      <c r="G13" s="49"/>
+      <c r="H13" s="33"/>
+    </row>
+    <row r="14" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B14" s="18" t="s">
-        <v>11</v>
+        <v>41</v>
       </c>
       <c r="C14" s="18">
+        <v>3</v>
+      </c>
+      <c r="D14" s="18">
         <v>1</v>
       </c>
-      <c r="D14" s="47"/>
-      <c r="E14" s="48"/>
-      <c r="F14" s="49"/>
-      <c r="G14" s="33"/>
-    </row>
-    <row r="15" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B15" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="C15" s="18">
+      <c r="E14" s="47"/>
+      <c r="F14" s="48"/>
+      <c r="G14" s="49"/>
+      <c r="H14" s="33"/>
+    </row>
+    <row r="15" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B15" s="23" t="s">
+        <v>38</v>
+      </c>
+      <c r="C15" s="23">
+        <v>3</v>
+      </c>
+      <c r="D15" s="18">
         <v>1</v>
       </c>
-      <c r="D15" s="50"/>
-      <c r="E15" s="51"/>
-      <c r="F15" s="52"/>
-      <c r="G15" s="34"/>
+      <c r="E15" s="50"/>
+      <c r="F15" s="51"/>
+      <c r="G15" s="52"/>
+      <c r="H15" s="34"/>
     </row>
   </sheetData>
   <mergeCells count="8">
-    <mergeCell ref="D2:G2"/>
-    <mergeCell ref="D6:D8"/>
-    <mergeCell ref="F6:F11"/>
-    <mergeCell ref="G3:G15"/>
-    <mergeCell ref="D3:F5"/>
-    <mergeCell ref="D12:F15"/>
-    <mergeCell ref="D9:D10"/>
-    <mergeCell ref="E6:E10"/>
+    <mergeCell ref="E2:H2"/>
+    <mergeCell ref="E6:E8"/>
+    <mergeCell ref="G6:G11"/>
+    <mergeCell ref="H3:H15"/>
+    <mergeCell ref="E3:G5"/>
+    <mergeCell ref="E12:G15"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="F6:F10"/>
   </mergeCells>
-  <conditionalFormatting sqref="C3:C5">
+  <conditionalFormatting sqref="D3:D5">
     <cfRule type="colorScale" priority="25">
       <colorScale>
         <cfvo type="min"/>
@@ -2048,7 +2102,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C3:C8 C12:C15">
+  <conditionalFormatting sqref="D3:D8 D12:D15">
     <cfRule type="colorScale" priority="18">
       <colorScale>
         <cfvo type="min"/>
@@ -2068,7 +2122,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C3:C15">
+  <conditionalFormatting sqref="D3:D15">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -2078,7 +2132,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C6:C8">
+  <conditionalFormatting sqref="D6:D8">
     <cfRule type="colorScale" priority="24">
       <colorScale>
         <cfvo type="min"/>
@@ -2090,7 +2144,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C9">
+  <conditionalFormatting sqref="D9">
     <cfRule type="colorScale" priority="8">
       <colorScale>
         <cfvo type="min"/>
@@ -2102,7 +2156,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C9:C10">
+  <conditionalFormatting sqref="D9:D10">
     <cfRule type="colorScale" priority="5">
       <colorScale>
         <cfvo type="min"/>
@@ -2122,7 +2176,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C10">
+  <conditionalFormatting sqref="D10">
     <cfRule type="colorScale" priority="7">
       <colorScale>
         <cfvo type="min"/>
@@ -2134,7 +2188,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C11">
+  <conditionalFormatting sqref="D11">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -2164,7 +2218,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C12:C15">
+  <conditionalFormatting sqref="D12:D15">
     <cfRule type="colorScale" priority="20">
       <colorScale>
         <cfvo type="min"/>
@@ -2179,7 +2233,7 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <ignoredErrors>
-    <ignoredError sqref="F6 D12 D3 D9 D6" formulaRange="1"/>
+    <ignoredError sqref="G6 E12 E3 E9 E6" formulaRange="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>